<commit_message>
Import template adds Player Email and Player Phone columns
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/coach/CourtSense_Import_Template.xlsx
+++ b/coach/CourtSense_Import_Template.xlsx
@@ -582,7 +582,7 @@
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>ROSTER          Your players. This is the only required sheet. First name, last name, and grad year are the only required columns. You can also bring in jersey, TruVolley rating, height, standing reach, position, side, hand, and both parents with name, email, and phone.</t>
+          <t>ROSTER          Your players. This is the only required sheet. First name, last name, and grad year are the only required columns. You can also bring in jersey, TruVolley rating, height, standing reach, position, side, hand, the player's own email and cell phone, and both parents with name, email, and phone.</t>
         </is>
       </c>
     </row>
@@ -700,7 +700,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P5"/>
+  <dimension ref="A1:R5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -716,6 +716,8 @@
     <col width="18" customWidth="1" min="11" max="11"/>
     <col width="24" customWidth="1" min="12" max="12"/>
     <col width="16" customWidth="1" min="13" max="13"/>
+    <col width="26" customWidth="1" min="17" max="17"/>
+    <col width="16" customWidth="1" min="18" max="18"/>
   </cols>
   <sheetData>
     <row r="1" ht="21" customHeight="1">
@@ -813,6 +815,16 @@
           <t>Parent 2 Phone</t>
         </is>
       </c>
+      <c r="Q4" s="7" t="inlineStr">
+        <is>
+          <t>Player Email</t>
+        </is>
+      </c>
+      <c r="R4" s="7" t="inlineStr">
+        <is>
+          <t>Player Phone</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="8" t="inlineStr">
@@ -880,8 +892,8 @@
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A1:P1"/>
-    <mergeCell ref="A2:P2"/>
+    <mergeCell ref="A1:R1"/>
+    <mergeCell ref="A2:R2"/>
   </mergeCells>
   <dataValidations count="4">
     <dataValidation sqref="C5:C300" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">

</xml_diff>